<commit_message>
Refactor image fetching and rendering logic: - Change image URL fetching to download image bytes from OneDrive via Graph API. - Update caching mechanism to store image bytes instead of URLs. - Modify image rendering to handle bytes directly, removing reliance on URL tuples. - Improve error handling and timeout settings for API requests. - Clean up code by removing unused variables and simplifying logic for displaying images.
</commit_message>
<xml_diff>
--- a/Data/Coordinates sheet.xlsx
+++ b/Data/Coordinates sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f324605ffb35608a/Archaeology/PhD/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="11_3187953798CD378BAAC55F735C773309FC0B06EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35A6E9B4-A5E5-4B91-AF5A-CB92A87EA750}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="11_3187953798CD378BAAC55F735C773309FC0B06EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44AAB5B5-6E66-4127-8E1F-3C57DF8D4B4F}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Archaeology Sites Coord" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="792" uniqueCount="240">
   <si>
     <t>n</t>
   </si>
@@ -742,6 +742,9 @@
   </si>
   <si>
     <t>La Zarcita</t>
+  </si>
+  <si>
+    <t>Cueva de la Mora</t>
   </si>
 </sst>
 </file>
@@ -1031,7 +1034,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1392,7 +1395,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.5546875" style="6" bestFit="1" customWidth="1"/>
@@ -2148,6 +2151,23 @@
       </c>
       <c r="E44" s="1">
         <v>37.771180200000003</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="7">
+        <v>44</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="C45" s="16" t="s">
+        <v>230</v>
+      </c>
+      <c r="D45" s="3">
+        <v>6.7422301999999998</v>
+      </c>
+      <c r="E45" s="1">
+        <v>37.917215599999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update data files: add missing site names and clean up Excel data
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/Coordinates sheet.xlsx
+++ b/Data/Coordinates sheet.xlsx
@@ -727,7 +727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6.5546875" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
@@ -1694,19 +1694,19 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MLin DEC</t>
+          <t>Carmona</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Upper Guadalquivir</t>
+          <t>Lower Guadalquivir</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>3.6344574</v>
+        <v>5.641821</v>
       </c>
       <c r="E46" t="n">
-        <v>38.0930873</v>
+        <v>37.471274</v>
       </c>
     </row>
     <row r="47">
@@ -1715,19 +1715,19 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MJ DEC</t>
+          <t>Constantina</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Upper Guadalquivir</t>
+          <t>Lower Guadalquivir</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>3.7892566</v>
+        <v>5.6191151</v>
       </c>
       <c r="E47" t="n">
-        <v>37.7741332</v>
+        <v>37.8722721</v>
       </c>
     </row>
     <row r="48">
@@ -1736,82 +1736,19 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MUbe DEC</t>
+          <t>El Coronil</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Upper Guadalquivir</t>
+          <t>Lower Guadalquivir</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>3.3711</v>
+        <v>5.6337983</v>
       </c>
       <c r="E48" t="n">
-        <v>38.0137</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>UGR Department DEC</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Subbaetic</t>
-        </is>
-      </c>
-      <c r="D49" t="n">
-        <v>3.5965129</v>
-      </c>
-      <c r="E49" t="n">
-        <v>37.1907621</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>MCor DEC</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Middle Guadalquivir</t>
-        </is>
-      </c>
-      <c r="D50" t="n">
-        <v>4.777926</v>
-      </c>
-      <c r="E50" t="n">
-        <v>37.881909</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>MAlm DEC</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Southeast</t>
-        </is>
-      </c>
-      <c r="D51" t="n">
-        <v>2.4556464</v>
-      </c>
-      <c r="E51" t="n">
-        <v>36.8385874</v>
+        <v>37.0793653</v>
       </c>
     </row>
   </sheetData>

</xml_diff>